<commit_message>
fix: map Hisui Challenges to perfectly 1-to-1 route unlock sequence
- Refactored the 'Challenges' sheet to programmatically generate one sequence-locked Challenge for every single route present in the 'Paths' sheet
- Challenge requisites are now tied dynamically to the preceding route (e.g. Defeating Pokemon in the route, visiting the Daycare, or defeating a Gym/Noble) to explicitly unlock the next route in the chronological path
- Preserved the 4 extra challenge chains (Space-Time Distortions, Wisps, Unown, Legends) at the bottom of the sheet as originally requested

Co-authored-by: lsampaio1337-beep <246645260+lsampaio1337-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Hisui_Paths.xlsx
+++ b/Hisui_Paths.xlsx
@@ -11901,7 +11901,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11929,12 +11929,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Defeat Gym - Kleavor</t>
+          <t>Defeat 10 Pokemon in Jubilife Village</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Unlock Crimson Mirelands (Golden Lowlands North)</t>
+          <t>Unlock Jubilife Village Daycare</t>
         </is>
       </c>
     </row>
@@ -11946,12 +11946,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Defeat Gym - Lilligant</t>
+          <t>Visit Jubilife Village Daycare</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Unlock Cobalt Coastlands (Crossing Slope)</t>
+          <t>Unlock Aspiration Hill</t>
         </is>
       </c>
     </row>
@@ -11963,12 +11963,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Defeat Gym - Arcanine</t>
+          <t>Defeat 10 Pokemon in Aspiration Hill</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Unlock Coronet Highlands (Celestica Trail)</t>
+          <t>Unlock Horseshoe Plains</t>
         </is>
       </c>
     </row>
@@ -11980,12 +11980,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Defeat Gym - Electrode</t>
+          <t>Defeat 10 Pokemon in Horseshoe Plains</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Unlock Alabaster Icelands (Whiteout Valley)</t>
+          <t>Unlock Horseshoe Plains (Fishing Spot)</t>
         </is>
       </c>
     </row>
@@ -11997,12 +11997,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Defeat Gym - Avalugg</t>
+          <t>Defeat 10 Pokemon in Horseshoe Plains (Fishing Spot) (Water)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Unlock Clan Leaders Battles</t>
+          <t>Unlock Floaro Gardens</t>
         </is>
       </c>
     </row>
@@ -12014,12 +12014,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Defeat Gym - Warden Ingo</t>
+          <t>Defeat 10 Pokemon in Floaro Gardens</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Unlock Late Game Exploring (Worn Bridge)</t>
+          <t>Unlock Deertrack Path</t>
         </is>
       </c>
     </row>
@@ -12031,248 +12031,1761 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Complete Late Game Exploring</t>
+          <t>Defeat 10 Pokemon in Deertrack Path</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Unlock Hisui Pokemon League</t>
+          <t>Unlock Deertrack Heights</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Extra Challenge 1-1</t>
+          <t>Challenge 8</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Defeat Gym - Kleavor</t>
+          <t>Defeat 10 Pokemon in Deertrack Heights</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Unlock Space-Time Distortion (Level 1)</t>
+          <t>Unlock Gym - Kleavor</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Extra Challenge 1-2</t>
+          <t>Challenge 9</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Defeat Gym - Lilligant</t>
+          <t>Defeat Gym - Kleavor</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Unlock Space-Time Distortion (Level 2)</t>
+          <t>Unlock Oreburrow Tunnel</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Extra Challenge 1-3</t>
+          <t>Challenge 10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Defeat Gym - Avalugg</t>
+          <t>Defeat 10 Pokemon in Oreburrow Tunnel</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Unlock Space-Time Distortion (Level 3)</t>
+          <t>Unlock Nature’s Pantry</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Extra Challenge 1-4</t>
+          <t>Challenge 11</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Defeat Hisui Pokemon League</t>
+          <t>Defeat 10 Pokemon in Nature’s Pantry</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Unlock Space-Time Distortion (Max Level)</t>
+          <t>Unlock The Heartwood North</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Extra Challenge 2-1</t>
+          <t>Challenge 12</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Capture 10 Ghost Type Pokemon</t>
+          <t>Defeat 10 Pokemon in The Heartwood North</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Unlock Wisp Encounter: Gastly / Haunter</t>
+          <t>Unlock The Heartwood South</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Extra Challenge 2-2</t>
+          <t>Challenge 13</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Defeat Gym - Arcanine &amp; Capture 30 Ghost Type Pokemon</t>
+          <t>Defeat 10 Pokemon in The Heartwood South</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Unlock Wisp Encounter: Misdreavus / Mismagius</t>
+          <t>Unlock The Heartwood South (Fishing Spot)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Extra Challenge 2-3</t>
+          <t>Challenge 14</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Defeat Hisui Pokemon League &amp; Capture 50 Ghost Type Pokemon</t>
+          <t>Defeat 10 Pokemon in The Heartwood South (Fishing Spot) (Water)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Unlock Spiritomb Encounter</t>
+          <t>Unlock Golden Lowlands North</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Extra Challenge 3-1</t>
+          <t>Challenge 15</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Capture 10 different species in Crimson Mirelands</t>
+          <t>Defeat 10 Pokemon in Golden Lowlands North</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Unlock Unown Ruins (A-F)</t>
+          <t>Unlock Golden Lowlands North (Fishing Spot)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Extra Challenge 3-2</t>
+          <t>Challenge 16</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Capture 10 different species in Cobalt Coastlands</t>
+          <t>Defeat 10 Pokemon in Golden Lowlands North (Fishing Spot) (Water)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Unlock Unown Ruins (G-L)</t>
+          <t>Unlock Golden Lowlands South</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Extra Challenge 3-3</t>
+          <t>Challenge 17</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Capture 10 different species in Coronet Highlands</t>
+          <t>Defeat 10 Pokemon in Golden Lowlands South</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Unlock Unown Ruins (M-S)</t>
+          <t>Unlock Golden Lowlands South (Fishing Spot)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Extra Challenge 3-4</t>
+          <t>Challenge 18</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Capture 10 different species in Alabaster Icelands</t>
+          <t>Defeat 10 Pokemon in Golden Lowlands South (Fishing Spot) (Water)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Unlock Unown Ruins (T-Z, !, ?)</t>
+          <t>Unlock Gapejaw Bog North</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Extra Challenge 4-1</t>
+          <t>Challenge 19</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Capture Uxie, Mesprit, Azelf</t>
+          <t>Defeat 10 Pokemon in Gapejaw Bog North</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Unlock Red Chain Item</t>
+          <t>Unlock Gapejaw Bog North (Fishing Spot)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Extra Challenge 4-2</t>
+          <t>Challenge 20</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Defeat Hisui Pokemon League &amp; Hold Red Chain</t>
+          <t>Defeat 10 Pokemon in Gapejaw Bog North (Fishing Spot) (Water)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Unlock Dialga / Palkia Battle</t>
+          <t>Unlock Gapejaw Bog South</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>Challenge 21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Gapejaw Bog South</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Unlock Gapejaw Bog South (Fishing Spot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Challenge 22</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Gapejaw Bog South (Fishing Spot) (Water)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Unlock Gym - Lilligant</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Challenge 23</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Defeat Gym - Lilligant</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Unlock Ursa's Ring</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Challenge 24</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Ursa's Ring</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Unlock Sludge Mound</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Challenge 25</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Sludge Mound</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Unlock Scarlet Bog</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Challenge 26</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Scarlet Bog</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Unlock Bolderoll Slope</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Challenge 27</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Bolderoll Slope</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Unlock Holm of Trials</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Challenge 28</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Holm of Trials</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Unlock Holm of Trials (Fishing Spot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Challenge 29</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Holm of Trials (Fishing Spot) (Water)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Unlock Crossing Slope</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Challenge 30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Crossing Slope</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Unlock Bathers' Lagoon</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Challenge 31</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Bathers' Lagoon</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Unlock Bathers' Lagoon (Fishing Spot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Challenge 32</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Bathers' Lagoon (Fishing Spot) (Water)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Unlock Castaway Shore</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Challenge 33</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Castaway Shore</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Unlock Castaway Shore (Fishing Spot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Challenge 34</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Castaway Shore (Fishing Spot) (Water)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Unlock Gym - Arcanine</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Challenge 35</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Defeat Gym - Arcanine</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Unlock Veilstone Cape</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Challenge 36</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Veilstone Cape</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Unlock Tranquility Cove</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Challenge 37</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Tranquility Cove</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Unlock Tranquility Cove (Fishing Spot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Challenge 38</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Tranquility Cove (Fishing Spot) (Water)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Unlock Islespy Shore</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Challenge 39</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Islespy Shore</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Unlock Islespy Shore (Fishing Spot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Challenge 40</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Islespy Shore (Fishing Spot) (Water)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Unlock Seagrass Haven</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Challenge 41</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Seagrass Haven</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Unlock Deadwood Haunt</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Challenge 42</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Deadwood Haunt</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Unlock Firespit Island</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Challenge 43</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Firespit Island</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Unlock Spring Path</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Challenge 44</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Spring Path</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Unlock Spring Path (Fishing Spot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Challenge 45</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Spring Path (Fishing Spot) (Water)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Unlock Celestica Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Challenge 46</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Celestica Trail</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Unlock Celestica Ruins</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Challenge 47</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Celestica Ruins</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Unlock Gym - Electrode</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Challenge 48</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Defeat Gym - Electrode</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Unlock Clamberclaw Cliffs</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Challenge 49</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Clamberclaw Cliffs</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Unlock Sacred Plaza</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Challenge 50</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Sacred Plaza</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Unlock Stonetooth Rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Challenge 51</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Stonetooth Rows</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Unlock Primeval Grotto</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Challenge 52</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Primeval Grotto</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Unlock Primeval Grotto (Fishing Spot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Challenge 53</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Primeval Grotto (Fishing Spot) (Water)</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Unlock Coronet Highlands</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Challenge 54</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Coronet Highlands</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Unlock Fabled Spring</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Challenge 55</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Fabled Spring</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Unlock Fabled Spring (Fishing Spot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Challenge 56</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Fabled Spring (Fishing Spot) (Water)</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Unlock Whiteout Valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Challenge 57</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Whiteout Valley</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Unlock Bonechill Wastes North</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Challenge 58</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Bonechill Wastes North</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Unlock Bonechill Wastes South</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Challenge 59</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Bonechill Wastes South</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Unlock Gym - Avalugg</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Challenge 60</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Defeat Gym - Avalugg</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Unlock Icebound Falls</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Challenge 61</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Icebound Falls</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Unlock Arena's Approach</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Challenge 62</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Arena's Approach</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Unlock Glacier Terrace</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Challenge 63</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Glacier Terrace</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Unlock Snowpoint Temple</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Challenge 64</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Snowpoint Temple</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Unlock Heart's Crag</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Challenge 65</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Heart's Crag</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Unlock Heart's Crag (Fishing Spot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Challenge 66</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Heart's Crag (Fishing Spot) (Water)</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Unlock Gym - Clan Leader Adaman</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Challenge 67</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Defeat Gym - Clan Leader Adaman</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Unlock Gym - Clan Leader Irida</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Challenge 68</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Defeat Gym - Clan Leader Irida</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Unlock Gym - Warden Ingo</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Challenge 69</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Defeat Gym - Warden Ingo</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Unlock Worn Bridge</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Challenge 70</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Worn Bridge</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Unlock Worn Bridge (Fishing Spot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Challenge 71</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Worn Bridge (Fishing Spot) (Water)</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Unlock Droning Meadow</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Challenge 72</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Droning Meadow</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Unlock Grueling Grove</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Challenge 73</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Grueling Grove</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Unlock Sandgem Flats North</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Challenge 74</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Sandgem Flats North</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Unlock Sandgem Flats North (Fishing Spot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Challenge 75</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Sandgem Flats North (Fishing Spot) (Water)</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Unlock Sandgem Flats South</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Challenge 76</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Sandgem Flats South</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Unlock Sandgem Flats South (Fishing Spot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Challenge 77</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Sandgem Flats South (Fishing Spot) (Water)</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Unlock Ginkgo Landing</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Challenge 78</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Ginkgo Landing</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Unlock Ginkgo Landing (Fishing Spot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Challenge 79</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Ginkgo Landing (Fishing Spot) (Water)</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Unlock Ramanas Island North</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Challenge 80</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Ramanas Island North</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Unlock Ramanas Island North (Fishing Spot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Challenge 81</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Ramanas Island North (Fishing Spot) (Water)</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Unlock Ramanas Island South</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Challenge 82</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Ramanas Island South</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Unlock Ramanas Island South (Fishing Spot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Challenge 83</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Ramanas Island South (Fishing Spot) (Water)</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Unlock Obsidian Falls</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Challenge 84</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Obsidian Falls</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Unlock Obsidian Falls (Fishing Spot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Challenge 85</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Obsidian Falls (Fishing Spot) (Water)</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Unlock Lake Verity</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Challenge 86</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Lake Verity</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Unlock Lake Verity (Fishing Spot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Challenge 87</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Lake Verity (Fishing Spot) (Water)</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Unlock Lake Valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Challenge 88</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Lake Valor</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Unlock Lake Valor (Fishing Spot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Challenge 89</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Lake Valor (Fishing Spot) (Water)</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Unlock Wayward Cave</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Challenge 90</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Wayward Cave</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Unlock Wayward Cave (Fishing Spot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Challenge 91</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Wayward Cave (Fishing Spot) (Water)</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Unlock Cloudpool Ridge North</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Challenge 92</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Cloudpool Ridge North</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Unlock Cloudpool Ridge South</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Challenge 93</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Cloudpool Ridge South</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Unlock Seaside Hollow</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Challenge 94</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Seaside Hollow</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Unlock Shrouded Ruins</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Challenge 95</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Shrouded Ruins</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Unlock Space-Time Distortion</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Challenge 96</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Defeat 10 Pokemon in Space-Time Distortion</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Unlock Hisui Pokemon League</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Extra Challenge 1-1</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Defeat Gym - Kleavor</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Unlock Space-Time Distortion (Level 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Extra Challenge 1-2</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Defeat Gym - Lilligant</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Unlock Space-Time Distortion (Level 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Extra Challenge 1-3</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Defeat Gym - Avalugg</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Unlock Space-Time Distortion (Level 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Extra Challenge 1-4</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Defeat Hisui Pokemon League</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Unlock Space-Time Distortion (Max Level)</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Extra Challenge 2-1</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Capture 10 Ghost Type Pokemon</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Unlock Wisp Encounter: Gastly / Haunter</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Extra Challenge 2-2</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Defeat Gym - Arcanine &amp; Capture 30 Ghost Type Pokemon</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Unlock Wisp Encounter: Misdreavus / Mismagius</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Extra Challenge 2-3</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Defeat Hisui Pokemon League &amp; Capture 50 Ghost Type Pokemon</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Unlock Spiritomb Encounter</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Extra Challenge 3-1</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Capture 10 different species in Crimson Mirelands</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Unlock Unown Ruins (A-F)</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Extra Challenge 3-2</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Capture 10 different species in Cobalt Coastlands</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Unlock Unown Ruins (G-L)</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Extra Challenge 3-3</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Capture 10 different species in Coronet Highlands</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Unlock Unown Ruins (M-S)</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Extra Challenge 3-4</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Capture 10 different species in Alabaster Icelands</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Unlock Unown Ruins (T-Z, !, ?)</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Extra Challenge 4-1</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Capture Uxie, Mesprit, Azelf</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Unlock Red Chain Item</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Extra Challenge 4-2</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Defeat Hisui Pokemon League &amp; Hold Red Chain</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Unlock Dialga / Palkia Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
           <t>Extra Challenge 4-3</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B111" t="inlineStr">
         <is>
           <t>Complete Hisui Pokedex (All Sheets)</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C111" t="inlineStr">
         <is>
           <t>Unlock Arceus Battle (Temple of Sinnoh)</t>
         </is>

</xml_diff>